<commit_message>
fix(qa): replace phantom BUG-10 with real 422 server validation bug, fix TC-05 boundary fixtures, wire dynamic Postman variables and isolate top 3 PM issues
</commit_message>
<xml_diff>
--- a/kvitto_tables.xlsx
+++ b/kvitto_tables.xlsx
@@ -679,10 +679,10 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1. Нижняя граница: ввести 2 символа («Ян Ли»)
-2. Околопредельная верхняя: ввести 99 символов
-3. Точная верхняя граница: ввести ровно 100 символов
-4. Выход за границу: ввести 101 символ</t>
+          <t>1. Нижняя граница: ввести 2 символа («Ян»)
+2. Околопредельная: строка 99 символов («Александр-» + 88 букв «а» + «в»)
+3. Точная верхняя граница: строка 100 символов («Александр-» + 89 букв «а» + «в»)
+4. Выход за границу: строка 101 символ («Александр-» + 90 букв «а» + «в»)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Отправка чека на альтернативный email (receipt_email)</t>
+          <t>Отображение серверных ошибок валидации при неверном коде страны в телефоне</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -875,15 +875,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1. Заполнить основной Email: «main@example.com»
-2. Установить чекбокс «Отправить чек на другой email»
-3. В появившееся поле ввести «other@company.ru»
-4. Заполнить остальные обязательные поля и нажать «Оплатить»</t>
+          <t>1. Заполнить имя и email
+2. В поле «Телефон» ввести номер с кодом США: «+1 999 123-45-67» (проходит клиентскую проверку длины)
+3. Нажать «Оплатить»</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>В запросе к API передается receipt_email: 'other@company.ru'. Сервер сохраняет данный адрес. На экране успеха в поле «Чек на» отображается «other@company.ru».</t>
+          <t>Бэкенд возвращает 422 validation_error. Ошибка отображается под полем «Телефон» (п. 2 ТЗ: ошибки сервера показываются под соответствующими полями).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -893,7 +892,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>BUG-10, BUG-15</t>
+          <t>BUG-10</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1406,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Экран успеха: Поле «Чек на» пустое, если не был указан альтернативный email</t>
+          <t>Валидация: Фронтенд не отображает серверные ошибки полей (выводится только общий баннер)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1417,33 +1416,33 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1. Заполнить форму с основным email: «user@example.com»
-2. Чекбокс «Отправить чек на другой email» не включать
-3. Нажать кнопку «Оплатить» и дождаться экрана успеха</t>
+          <t>1. Заполнить имя и email
+2. В поле «Телефон» ввести номер с кодом США: «+1 999 123-45-67»
+3. Нажать «Оплатить»</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>В строке «Чек на» отображается основной адрес покупателя: «user@example.com» (по ТЗ: «адрес, на который придёт чек»).</t>
+          <t>Серверная ошибка валидации отображается под полем «Телефон» (по ТЗ: ошибки сервера показываются под соответствующими полями).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Строка «Чек на» остаётся пустой.</t>
+          <t>Фронтенд игнорирует объект fields и показывает только общий баннер «Что-то пошло не так». Поле не подсвечивается.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Средняя</t>
+          <t>Высокая</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Средний</t>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="I11" s="3">
-        <f>HYPERLINK("https://github.com/msmr14/kvittoqademo/blob/main/screenshots/BUG-10.png", "скриншот экрана «Платёж создан» с пустой строкой «Чек на» ↗")</f>
+        <f>HYPERLINK("https://github.com/msmr14/kvittoqademo/blob/main/screenshots/BUG-10.png", "скриншот формы с общим баннером вместо ошибки под полем ↗")</f>
         <v/>
       </c>
     </row>

</xml_diff>